<commit_message>
Kirsten added chl-a ggpairs analysis
</commit_message>
<xml_diff>
--- a/DataRaw/NARWPercentOccur_Chla_8daySummary_080726.xlsx
+++ b/DataRaw/NARWPercentOccur_Chla_8daySummary_080726.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kirsten/Desktop/KirstensWork/NARW Consortium 2025/NARWCon_2025/DataRaw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDAEACF3-28CE-C048-A718-4F78254B3062}" xr6:coauthVersionLast="40" xr6:coauthVersionMax="40" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B581259C-38F9-DC4B-BA4A-2494007091F3}" xr6:coauthVersionLast="40" xr6:coauthVersionMax="40" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30400" yWindow="-500" windowWidth="36980" windowHeight="20920" xr2:uid="{83087B85-8CB4-5A41-BEF3-B3A02C17795A}"/>
+    <workbookView xWindow="30500" yWindow="-2020" windowWidth="36980" windowHeight="20920" xr2:uid="{83087B85-8CB4-5A41-BEF3-B3A02C17795A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -86,18 +86,12 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.59999389629810485"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -115,10 +109,10 @@
   <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="14" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -7359,26 +7353,26 @@
         <v>11.19006795</v>
       </c>
     </row>
-    <row r="302" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A302" s="2">
+    <row r="302" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A302" s="4">
         <v>42740</v>
       </c>
-      <c r="B302" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C302" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D302" s="3">
+      <c r="B302" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C302" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="D302" s="5">
         <v>5</v>
       </c>
-      <c r="E302" s="3" t="s">
+      <c r="E302" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="F302" s="3" t="s">
+      <c r="F302" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="G302" s="3">
+      <c r="G302" s="5">
         <v>9.2352078800000008</v>
       </c>
     </row>
@@ -7590,209 +7584,209 @@
       </c>
     </row>
     <row r="312" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A312" s="4">
+      <c r="A312" s="2">
         <v>42772</v>
       </c>
-      <c r="B312" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C312" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="D312" s="5">
-        <v>8</v>
-      </c>
-      <c r="E312" s="5">
-        <v>0</v>
-      </c>
-      <c r="F312" s="5">
-        <v>0</v>
-      </c>
-      <c r="G312" s="5">
+      <c r="B312" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C312" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D312" s="3">
+        <v>8</v>
+      </c>
+      <c r="E312" s="3">
+        <v>0</v>
+      </c>
+      <c r="F312" s="3">
+        <v>0</v>
+      </c>
+      <c r="G312" s="3">
         <v>2.84956875</v>
       </c>
     </row>
     <row r="313" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A313" s="4">
+      <c r="A313" s="2">
         <v>42772</v>
       </c>
-      <c r="B313" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C313" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="D313" s="5">
-        <v>8</v>
-      </c>
-      <c r="E313" s="5">
-        <v>0</v>
-      </c>
-      <c r="F313" s="5">
-        <v>0</v>
-      </c>
-      <c r="G313" s="5">
+      <c r="B313" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C313" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D313" s="3">
+        <v>8</v>
+      </c>
+      <c r="E313" s="3">
+        <v>0</v>
+      </c>
+      <c r="F313" s="3">
+        <v>0</v>
+      </c>
+      <c r="G313" s="3">
         <v>1.9819289200000001</v>
       </c>
     </row>
     <row r="314" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A314" s="4">
+      <c r="A314" s="2">
         <v>42772</v>
       </c>
-      <c r="B314" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C314" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="D314" s="5">
-        <v>8</v>
-      </c>
-      <c r="E314" s="5">
+      <c r="B314" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C314" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D314" s="3">
+        <v>8</v>
+      </c>
+      <c r="E314" s="3">
         <v>1</v>
       </c>
-      <c r="F314" s="5">
+      <c r="F314" s="3">
         <v>12.5</v>
       </c>
-      <c r="G314" s="5">
+      <c r="G314" s="3">
         <v>1.71705</v>
       </c>
     </row>
     <row r="315" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A315" s="4">
+      <c r="A315" s="2">
         <v>42780</v>
       </c>
-      <c r="B315" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C315" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="D315" s="5">
-        <v>8</v>
-      </c>
-      <c r="E315" s="5">
-        <v>0</v>
-      </c>
-      <c r="F315" s="5">
-        <v>0</v>
-      </c>
-      <c r="G315" s="5">
+      <c r="B315" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C315" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D315" s="3">
+        <v>8</v>
+      </c>
+      <c r="E315" s="3">
+        <v>0</v>
+      </c>
+      <c r="F315" s="3">
+        <v>0</v>
+      </c>
+      <c r="G315" s="3">
         <v>2.5603074399999999</v>
       </c>
     </row>
     <row r="316" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A316" s="4">
+      <c r="A316" s="2">
         <v>42780</v>
       </c>
-      <c r="B316" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C316" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="D316" s="5">
-        <v>8</v>
-      </c>
-      <c r="E316" s="5">
-        <v>0</v>
-      </c>
-      <c r="F316" s="5">
-        <v>0</v>
-      </c>
-      <c r="G316" s="5">
+      <c r="B316" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C316" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D316" s="3">
+        <v>8</v>
+      </c>
+      <c r="E316" s="3">
+        <v>0</v>
+      </c>
+      <c r="F316" s="3">
+        <v>0</v>
+      </c>
+      <c r="G316" s="3">
         <v>2.0980106699999999</v>
       </c>
     </row>
     <row r="317" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A317" s="4">
+      <c r="A317" s="2">
         <v>42780</v>
       </c>
-      <c r="B317" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C317" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="D317" s="5">
-        <v>8</v>
-      </c>
-      <c r="E317" s="5">
-        <v>0</v>
-      </c>
-      <c r="F317" s="5">
-        <v>0</v>
-      </c>
-      <c r="G317" s="5">
+      <c r="B317" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C317" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D317" s="3">
+        <v>8</v>
+      </c>
+      <c r="E317" s="3">
+        <v>0</v>
+      </c>
+      <c r="F317" s="3">
+        <v>0</v>
+      </c>
+      <c r="G317" s="3">
         <v>2.06284673</v>
       </c>
     </row>
     <row r="318" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A318" s="4">
+      <c r="A318" s="2">
         <v>42788</v>
       </c>
-      <c r="B318" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C318" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="D318" s="5">
-        <v>8</v>
-      </c>
-      <c r="E318" s="5">
-        <v>0</v>
-      </c>
-      <c r="F318" s="5">
-        <v>0</v>
-      </c>
-      <c r="G318" s="5">
+      <c r="B318" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C318" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D318" s="3">
+        <v>8</v>
+      </c>
+      <c r="E318" s="3">
+        <v>0</v>
+      </c>
+      <c r="F318" s="3">
+        <v>0</v>
+      </c>
+      <c r="G318" s="3">
         <v>1.8638284899999999</v>
       </c>
     </row>
     <row r="319" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A319" s="4">
+      <c r="A319" s="2">
         <v>42788</v>
       </c>
-      <c r="B319" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C319" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="D319" s="5">
-        <v>8</v>
-      </c>
-      <c r="E319" s="5">
-        <v>0</v>
-      </c>
-      <c r="F319" s="5">
-        <v>0</v>
-      </c>
-      <c r="G319" s="5">
+      <c r="B319" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C319" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D319" s="3">
+        <v>8</v>
+      </c>
+      <c r="E319" s="3">
+        <v>0</v>
+      </c>
+      <c r="F319" s="3">
+        <v>0</v>
+      </c>
+      <c r="G319" s="3">
         <v>1.43252037</v>
       </c>
     </row>
     <row r="320" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A320" s="4">
+      <c r="A320" s="2">
         <v>42788</v>
       </c>
-      <c r="B320" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C320" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="D320" s="5">
-        <v>8</v>
-      </c>
-      <c r="E320" s="5">
-        <v>0</v>
-      </c>
-      <c r="F320" s="5">
-        <v>0</v>
-      </c>
-      <c r="G320" s="5">
+      <c r="B320" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C320" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D320" s="3">
+        <v>8</v>
+      </c>
+      <c r="E320" s="3">
+        <v>0</v>
+      </c>
+      <c r="F320" s="3">
+        <v>0</v>
+      </c>
+      <c r="G320" s="3">
         <v>1.48917498</v>
       </c>
     </row>
@@ -9384,22 +9378,22 @@
       </c>
     </row>
     <row r="390" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A390" s="4">
+      <c r="A390" s="2">
         <v>42980</v>
       </c>
-      <c r="B390" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C390" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="D390" s="5">
-        <v>8</v>
-      </c>
-      <c r="E390" s="5">
-        <v>0</v>
-      </c>
-      <c r="F390" s="5">
+      <c r="B390" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C390" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D390" s="3">
+        <v>8</v>
+      </c>
+      <c r="E390" s="3">
+        <v>0</v>
+      </c>
+      <c r="F390" s="3">
         <v>0</v>
       </c>
       <c r="G390">
@@ -9407,22 +9401,22 @@
       </c>
     </row>
     <row r="391" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A391" s="4">
+      <c r="A391" s="2">
         <v>42980</v>
       </c>
-      <c r="B391" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C391" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="D391" s="5">
-        <v>8</v>
-      </c>
-      <c r="E391" s="5">
-        <v>0</v>
-      </c>
-      <c r="F391" s="5">
+      <c r="B391" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C391" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D391" s="3">
+        <v>8</v>
+      </c>
+      <c r="E391" s="3">
+        <v>0</v>
+      </c>
+      <c r="F391" s="3">
         <v>0</v>
       </c>
       <c r="G391">
@@ -9430,22 +9424,22 @@
       </c>
     </row>
     <row r="392" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A392" s="4">
+      <c r="A392" s="2">
         <v>42980</v>
       </c>
-      <c r="B392" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C392" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="D392" s="5">
-        <v>8</v>
-      </c>
-      <c r="E392" s="5">
-        <v>0</v>
-      </c>
-      <c r="F392" s="5">
+      <c r="B392" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C392" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D392" s="3">
+        <v>8</v>
+      </c>
+      <c r="E392" s="3">
+        <v>0</v>
+      </c>
+      <c r="F392" s="3">
         <v>0</v>
       </c>
       <c r="G392">
@@ -9453,22 +9447,22 @@
       </c>
     </row>
     <row r="393" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A393" s="4">
+      <c r="A393" s="2">
         <v>42988</v>
       </c>
-      <c r="B393" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C393" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="D393" s="5">
-        <v>8</v>
-      </c>
-      <c r="E393" s="5">
-        <v>0</v>
-      </c>
-      <c r="F393" s="5">
+      <c r="B393" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C393" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D393" s="3">
+        <v>8</v>
+      </c>
+      <c r="E393" s="3">
+        <v>0</v>
+      </c>
+      <c r="F393" s="3">
         <v>0</v>
       </c>
       <c r="G393">
@@ -9476,22 +9470,22 @@
       </c>
     </row>
     <row r="394" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A394" s="4">
+      <c r="A394" s="2">
         <v>42988</v>
       </c>
-      <c r="B394" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C394" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="D394" s="5">
-        <v>8</v>
-      </c>
-      <c r="E394" s="5">
-        <v>0</v>
-      </c>
-      <c r="F394" s="5">
+      <c r="B394" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C394" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D394" s="3">
+        <v>8</v>
+      </c>
+      <c r="E394" s="3">
+        <v>0</v>
+      </c>
+      <c r="F394" s="3">
         <v>0</v>
       </c>
       <c r="G394">
@@ -9499,22 +9493,22 @@
       </c>
     </row>
     <row r="395" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A395" s="4">
+      <c r="A395" s="2">
         <v>42988</v>
       </c>
-      <c r="B395" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C395" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="D395" s="5">
-        <v>8</v>
-      </c>
-      <c r="E395" s="5">
-        <v>0</v>
-      </c>
-      <c r="F395" s="5">
+      <c r="B395" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C395" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D395" s="3">
+        <v>8</v>
+      </c>
+      <c r="E395" s="3">
+        <v>0</v>
+      </c>
+      <c r="F395" s="3">
         <v>0</v>
       </c>
       <c r="G395">
@@ -9522,22 +9516,22 @@
       </c>
     </row>
     <row r="396" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A396" s="4">
+      <c r="A396" s="2">
         <v>42996</v>
       </c>
-      <c r="B396" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C396" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="D396" s="5">
-        <v>8</v>
-      </c>
-      <c r="E396" s="5">
-        <v>0</v>
-      </c>
-      <c r="F396" s="5">
+      <c r="B396" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C396" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D396" s="3">
+        <v>8</v>
+      </c>
+      <c r="E396" s="3">
+        <v>0</v>
+      </c>
+      <c r="F396" s="3">
         <v>0</v>
       </c>
       <c r="G396">
@@ -9545,22 +9539,22 @@
       </c>
     </row>
     <row r="397" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A397" s="4">
+      <c r="A397" s="2">
         <v>42996</v>
       </c>
-      <c r="B397" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C397" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="D397" s="5">
-        <v>8</v>
-      </c>
-      <c r="E397" s="5">
-        <v>0</v>
-      </c>
-      <c r="F397" s="5">
+      <c r="B397" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C397" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D397" s="3">
+        <v>8</v>
+      </c>
+      <c r="E397" s="3">
+        <v>0</v>
+      </c>
+      <c r="F397" s="3">
         <v>0</v>
       </c>
       <c r="G397">
@@ -9568,22 +9562,22 @@
       </c>
     </row>
     <row r="398" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A398" s="4">
+      <c r="A398" s="2">
         <v>42996</v>
       </c>
-      <c r="B398" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C398" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="D398" s="5">
-        <v>8</v>
-      </c>
-      <c r="E398" s="5">
-        <v>0</v>
-      </c>
-      <c r="F398" s="5">
+      <c r="B398" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C398" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D398" s="3">
+        <v>8</v>
+      </c>
+      <c r="E398" s="3">
+        <v>0</v>
+      </c>
+      <c r="F398" s="3">
         <v>0</v>
       </c>
       <c r="G398">
@@ -9591,22 +9585,22 @@
       </c>
     </row>
     <row r="399" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A399" s="4">
+      <c r="A399" s="2">
         <v>43004</v>
       </c>
-      <c r="B399" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C399" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="D399" s="5">
-        <v>8</v>
-      </c>
-      <c r="E399" s="5">
-        <v>0</v>
-      </c>
-      <c r="F399" s="5">
+      <c r="B399" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C399" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D399" s="3">
+        <v>8</v>
+      </c>
+      <c r="E399" s="3">
+        <v>0</v>
+      </c>
+      <c r="F399" s="3">
         <v>0</v>
       </c>
       <c r="G399">
@@ -9614,22 +9608,22 @@
       </c>
     </row>
     <row r="400" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A400" s="4">
+      <c r="A400" s="2">
         <v>43004</v>
       </c>
-      <c r="B400" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C400" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="D400" s="5">
-        <v>8</v>
-      </c>
-      <c r="E400" s="5">
-        <v>0</v>
-      </c>
-      <c r="F400" s="5">
+      <c r="B400" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C400" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D400" s="3">
+        <v>8</v>
+      </c>
+      <c r="E400" s="3">
+        <v>0</v>
+      </c>
+      <c r="F400" s="3">
         <v>0</v>
       </c>
       <c r="G400">
@@ -9637,22 +9631,22 @@
       </c>
     </row>
     <row r="401" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A401" s="4">
+      <c r="A401" s="2">
         <v>43004</v>
       </c>
-      <c r="B401" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C401" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="D401" s="5">
-        <v>8</v>
-      </c>
-      <c r="E401" s="5">
-        <v>0</v>
-      </c>
-      <c r="F401" s="5">
+      <c r="B401" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C401" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D401" s="3">
+        <v>8</v>
+      </c>
+      <c r="E401" s="3">
+        <v>0</v>
+      </c>
+      <c r="F401" s="3">
         <v>0</v>
       </c>
       <c r="G401">
@@ -9660,22 +9654,22 @@
       </c>
     </row>
     <row r="402" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A402" s="4">
+      <c r="A402" s="2">
         <v>43012</v>
       </c>
-      <c r="B402" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C402" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="D402" s="5">
-        <v>8</v>
-      </c>
-      <c r="E402" s="5">
-        <v>0</v>
-      </c>
-      <c r="F402" s="5">
+      <c r="B402" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C402" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D402" s="3">
+        <v>8</v>
+      </c>
+      <c r="E402" s="3">
+        <v>0</v>
+      </c>
+      <c r="F402" s="3">
         <v>0</v>
       </c>
       <c r="G402">
@@ -9683,22 +9677,22 @@
       </c>
     </row>
     <row r="403" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A403" s="4">
+      <c r="A403" s="2">
         <v>43012</v>
       </c>
-      <c r="B403" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C403" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="D403" s="5">
-        <v>8</v>
-      </c>
-      <c r="E403" s="5">
-        <v>0</v>
-      </c>
-      <c r="F403" s="5">
+      <c r="B403" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C403" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D403" s="3">
+        <v>8</v>
+      </c>
+      <c r="E403" s="3">
+        <v>0</v>
+      </c>
+      <c r="F403" s="3">
         <v>0</v>
       </c>
       <c r="G403">
@@ -9706,22 +9700,22 @@
       </c>
     </row>
     <row r="404" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A404" s="4">
+      <c r="A404" s="2">
         <v>43012</v>
       </c>
-      <c r="B404" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C404" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="D404" s="5">
-        <v>8</v>
-      </c>
-      <c r="E404" s="5">
-        <v>0</v>
-      </c>
-      <c r="F404" s="5">
+      <c r="B404" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C404" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D404" s="3">
+        <v>8</v>
+      </c>
+      <c r="E404" s="3">
+        <v>0</v>
+      </c>
+      <c r="F404" s="3">
         <v>0</v>
       </c>
       <c r="G404">
@@ -9729,22 +9723,22 @@
       </c>
     </row>
     <row r="405" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A405" s="4">
+      <c r="A405" s="2">
         <v>43020</v>
       </c>
-      <c r="B405" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C405" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="D405" s="5">
-        <v>8</v>
-      </c>
-      <c r="E405" s="5">
-        <v>0</v>
-      </c>
-      <c r="F405" s="5">
+      <c r="B405" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C405" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D405" s="3">
+        <v>8</v>
+      </c>
+      <c r="E405" s="3">
+        <v>0</v>
+      </c>
+      <c r="F405" s="3">
         <v>0</v>
       </c>
       <c r="G405">
@@ -9752,22 +9746,22 @@
       </c>
     </row>
     <row r="406" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A406" s="4">
+      <c r="A406" s="2">
         <v>43020</v>
       </c>
-      <c r="B406" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C406" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="D406" s="5">
-        <v>8</v>
-      </c>
-      <c r="E406" s="5">
-        <v>0</v>
-      </c>
-      <c r="F406" s="5">
+      <c r="B406" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C406" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D406" s="3">
+        <v>8</v>
+      </c>
+      <c r="E406" s="3">
+        <v>0</v>
+      </c>
+      <c r="F406" s="3">
         <v>0</v>
       </c>
       <c r="G406">
@@ -9775,22 +9769,22 @@
       </c>
     </row>
     <row r="407" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A407" s="4">
+      <c r="A407" s="2">
         <v>43020</v>
       </c>
-      <c r="B407" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C407" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="D407" s="5">
-        <v>8</v>
-      </c>
-      <c r="E407" s="5">
-        <v>0</v>
-      </c>
-      <c r="F407" s="5">
+      <c r="B407" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C407" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D407" s="3">
+        <v>8</v>
+      </c>
+      <c r="E407" s="3">
+        <v>0</v>
+      </c>
+      <c r="F407" s="3">
         <v>0</v>
       </c>
       <c r="G407">
@@ -9798,22 +9792,22 @@
       </c>
     </row>
     <row r="408" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A408" s="4">
+      <c r="A408" s="2">
         <v>43028</v>
       </c>
-      <c r="B408" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C408" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="D408" s="5">
-        <v>8</v>
-      </c>
-      <c r="E408" s="5">
-        <v>0</v>
-      </c>
-      <c r="F408" s="5">
+      <c r="B408" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C408" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D408" s="3">
+        <v>8</v>
+      </c>
+      <c r="E408" s="3">
+        <v>0</v>
+      </c>
+      <c r="F408" s="3">
         <v>0</v>
       </c>
       <c r="G408">
@@ -9821,22 +9815,22 @@
       </c>
     </row>
     <row r="409" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A409" s="4">
+      <c r="A409" s="2">
         <v>43028</v>
       </c>
-      <c r="B409" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C409" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="D409" s="5">
-        <v>8</v>
-      </c>
-      <c r="E409" s="5">
-        <v>0</v>
-      </c>
-      <c r="F409" s="5">
+      <c r="B409" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C409" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D409" s="3">
+        <v>8</v>
+      </c>
+      <c r="E409" s="3">
+        <v>0</v>
+      </c>
+      <c r="F409" s="3">
         <v>0</v>
       </c>
       <c r="G409">
@@ -9844,22 +9838,22 @@
       </c>
     </row>
     <row r="410" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A410" s="4">
+      <c r="A410" s="2">
         <v>43028</v>
       </c>
-      <c r="B410" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C410" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="D410" s="5">
-        <v>8</v>
-      </c>
-      <c r="E410" s="5">
-        <v>0</v>
-      </c>
-      <c r="F410" s="5">
+      <c r="B410" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C410" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D410" s="3">
+        <v>8</v>
+      </c>
+      <c r="E410" s="3">
+        <v>0</v>
+      </c>
+      <c r="F410" s="3">
         <v>0</v>
       </c>
       <c r="G410">
@@ -9867,22 +9861,22 @@
       </c>
     </row>
     <row r="411" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A411" s="4">
+      <c r="A411" s="2">
         <v>43036</v>
       </c>
-      <c r="B411" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C411" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="D411" s="5">
-        <v>8</v>
-      </c>
-      <c r="E411" s="5">
-        <v>0</v>
-      </c>
-      <c r="F411" s="5">
+      <c r="B411" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C411" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D411" s="3">
+        <v>8</v>
+      </c>
+      <c r="E411" s="3">
+        <v>0</v>
+      </c>
+      <c r="F411" s="3">
         <v>0</v>
       </c>
       <c r="G411">
@@ -9890,22 +9884,22 @@
       </c>
     </row>
     <row r="412" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A412" s="4">
+      <c r="A412" s="2">
         <v>43036</v>
       </c>
-      <c r="B412" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C412" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="D412" s="5">
-        <v>8</v>
-      </c>
-      <c r="E412" s="5">
-        <v>0</v>
-      </c>
-      <c r="F412" s="5">
+      <c r="B412" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C412" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D412" s="3">
+        <v>8</v>
+      </c>
+      <c r="E412" s="3">
+        <v>0</v>
+      </c>
+      <c r="F412" s="3">
         <v>0</v>
       </c>
       <c r="G412">
@@ -9913,22 +9907,22 @@
       </c>
     </row>
     <row r="413" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A413" s="4">
+      <c r="A413" s="2">
         <v>43036</v>
       </c>
-      <c r="B413" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C413" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="D413" s="5">
-        <v>8</v>
-      </c>
-      <c r="E413" s="5">
-        <v>0</v>
-      </c>
-      <c r="F413" s="5">
+      <c r="B413" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C413" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D413" s="3">
+        <v>8</v>
+      </c>
+      <c r="E413" s="3">
+        <v>0</v>
+      </c>
+      <c r="F413" s="3">
         <v>0</v>
       </c>
       <c r="G413">

</xml_diff>